<commit_message>
Cap nhat file mau bao gia moi: logo, ngan hang, QR, con dau, an cot trong
</commit_message>
<xml_diff>
--- a/templates/Bao_Gia_Mau_FIX.xlsx
+++ b/templates/Bao_Gia_Mau_FIX.xlsx
@@ -9,7 +9,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bao gia dai ly" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Bao gia dai ly'!$B$1:$J$45</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Bao gia dai ly'!$B$1:$J$52</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -475,6 +475,56 @@
     </pic>
     <clientData/>
   </twoCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>8</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="876300" cy="876300"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="2" name="Image 2" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId2"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>6</col>
+      <colOff>762000</colOff>
+      <row>45</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1333500" cy="1333500"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -701,7 +751,7 @@
     <row r="4" ht="19.5" customHeight="1">
       <c r="B4" s="14" t="inlineStr">
         <is>
-          <t xml:space="preserve">MST: </t>
+          <t>MST: 2601158676</t>
         </is>
       </c>
     </row>
@@ -1055,7 +1105,7 @@
       </c>
       <c r="D39" s="16" t="inlineStr">
         <is>
-          <t>……………………………………………………………</t>
+          <t>MB Bank - Chi Nhánh Thanh Thủy</t>
         </is>
       </c>
       <c r="I39" s="25" t="n"/>
@@ -1069,7 +1119,7 @@
       </c>
       <c r="D40" s="16" t="inlineStr">
         <is>
-          <t>……………………………………………………………</t>
+          <t>CÔNG TY TNHH ĐẦU TƯ VÀ XUẤT NHẬP KHẨU HƯNG THỊNH SMART</t>
         </is>
       </c>
       <c r="I40" s="28" t="n"/>
@@ -1083,7 +1133,7 @@
       </c>
       <c r="D41" s="16" t="inlineStr">
         <is>
-          <t>……………………………………………………………</t>
+          <t>8090688688</t>
         </is>
       </c>
       <c r="I41" s="30" t="n"/>

</xml_diff>

<commit_message>
Mau bao gia: bo vien QR, ten cty wrap khong bi cat
</commit_message>
<xml_diff>
--- a/templates/Bao_Gia_Mau_FIX.xlsx
+++ b/templates/Bao_Gia_Mau_FIX.xlsx
@@ -277,7 +277,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -347,15 +347,18 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1117,7 +1120,7 @@
           <t>Chủ tài khoản:</t>
         </is>
       </c>
-      <c r="D40" s="16" t="inlineStr">
+      <c r="D40" s="32" t="inlineStr">
         <is>
           <t>CÔNG TY TNHH ĐẦU TƯ VÀ XUẤT NHẬP KHẨU HƯNG THỊNH SMART</t>
         </is>

</xml_diff>

<commit_message>
TT thanh toan: moi dong 1 hang, nhan+noi dung sat nhau
</commit_message>
<xml_diff>
--- a/templates/Bao_Gia_Mau_FIX.xlsx
+++ b/templates/Bao_Gia_Mau_FIX.xlsx
@@ -1103,42 +1103,84 @@
     <row r="39" ht="21.75" customHeight="1">
       <c r="B39" s="24" t="inlineStr">
         <is>
-          <t>Ngân hàng:</t>
-        </is>
-      </c>
-      <c r="D39" s="16" t="inlineStr">
-        <is>
-          <t>MB Bank - Chi Nhánh Thanh Thủy</t>
-        </is>
-      </c>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="10"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve">Ngân hàng: </t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="10"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve">MB Bank - Chi Nhánh Thanh Thủy</t>
+          </r>
+        </is>
+      </c>
+      <c r="D39" s="16"/>
       <c r="I39" s="25" t="n"/>
       <c r="J39" s="27" t="n"/>
     </row>
     <row r="40" ht="21.75" customHeight="1">
       <c r="B40" s="24" t="inlineStr">
         <is>
-          <t>Chủ tài khoản:</t>
-        </is>
-      </c>
-      <c r="D40" s="32" t="inlineStr">
-        <is>
-          <t>CÔNG TY TNHH ĐẦU TƯ VÀ XUẤT NHẬP KHẨU HƯNG THỊNH SMART</t>
-        </is>
-      </c>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="10"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve">Chủ tài khoản: </t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="10"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve">CÔNG TY TNHH ĐẦU TƯ VÀ XUẤT NHẬP KHẨU HƯNG THỊNH SMART</t>
+          </r>
+        </is>
+      </c>
+      <c r="D40" s="16"/>
       <c r="I40" s="28" t="n"/>
       <c r="J40" s="29" t="n"/>
     </row>
     <row r="41" ht="21.75" customHeight="1">
       <c r="B41" s="24" t="inlineStr">
         <is>
-          <t>Số tài khoản:</t>
-        </is>
-      </c>
-      <c r="D41" s="16" t="inlineStr">
-        <is>
-          <t>8090688688</t>
-        </is>
-      </c>
+          <r>
+            <rPr>
+              <b/>
+              <sz val="10"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve">Số tài khoản: </t>
+          </r>
+          <r>
+            <rPr>
+              <sz val="10"/>
+              <color rgb="FF000000"/>
+              <rFont val="Times New Roman"/>
+              <family val="1"/>
+            </rPr>
+            <t xml:space="preserve">8090688688</t>
+          </r>
+        </is>
+      </c>
+      <c r="D41" s="16"/>
       <c r="I41" s="30" t="n"/>
       <c r="J41" s="31" t="n"/>
     </row>
@@ -1159,19 +1201,17 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="31">
     <mergeCell ref="B11:J11"/>
     <mergeCell ref="B24:H24"/>
     <mergeCell ref="B1:J1"/>
-    <mergeCell ref="D40:H40"/>
     <mergeCell ref="B38:J38"/>
     <mergeCell ref="G44:J44"/>
-    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="B39:H39"/>
     <mergeCell ref="B29:J29"/>
     <mergeCell ref="B34:J34"/>
     <mergeCell ref="B10:J10"/>
     <mergeCell ref="B9:J9"/>
-    <mergeCell ref="D41:H41"/>
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="B6:J6"/>
     <mergeCell ref="B30:J30"/>
@@ -1181,16 +1221,15 @@
     <mergeCell ref="B32:J32"/>
     <mergeCell ref="B35:J35"/>
     <mergeCell ref="B4:J4"/>
-    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="B40:H40"/>
     <mergeCell ref="I39:J41"/>
     <mergeCell ref="B23:H23"/>
     <mergeCell ref="B7:J7"/>
-    <mergeCell ref="D39:H39"/>
     <mergeCell ref="B3:J3"/>
     <mergeCell ref="B31:J31"/>
     <mergeCell ref="B27:J27"/>
     <mergeCell ref="B45:F45"/>
-    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="B41:H41"/>
     <mergeCell ref="B12:J12"/>
     <mergeCell ref="B2:J2"/>
     <mergeCell ref="G45:J45"/>

</xml_diff>